<commit_message>
test(calculators): implementing tests for 15.7 services
implementing tests for 15.7 services
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/14-electricity.xlsx
+++ b/packages/calculators/src/modules/test/14-electricity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B62A8979-0E92-8249-A018-5C435A43FC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F45D962-3960-A544-970D-8F89D1F49E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51400" yWindow="18340" windowWidth="28800" windowHeight="23520" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
+    <workbookView xWindow="51220" yWindow="18580" windowWidth="28800" windowHeight="23520" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
   <sheets>
     <sheet name="14.1.1.1" sheetId="3" r:id="rId1"/>
@@ -364,7 +364,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -455,7 +455,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -487,8 +487,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -856,7 +855,7 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="K1" s="20" t="s">
         <v>2</v>
       </c>
       <c r="M1" s="1" t="s">
@@ -864,10 +863,10 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="50" customHeight="1">
-      <c r="L2" s="21" t="s">
+      <c r="L2" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="N2" s="20" t="s">
         <v>38</v>
       </c>
     </row>
@@ -907,13 +906,13 @@
       <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" t="s">
         <v>42</v>
       </c>
       <c r="I4" t="s">
@@ -953,7 +952,7 @@
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="12">
-        <f>IF(ISBLANK(A5), "", VLOOKUP(B5, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" ref="E5:E13" si="0">IF(ISBLANK(A5), "", VLOOKUP(B5, $P$20:$T$28, 2, FALSE))</f>
         <v>0.68</v>
       </c>
       <c r="F5" s="12">
@@ -969,19 +968,19 @@
         <v>0.1</v>
       </c>
       <c r="I5" s="12">
-        <f>IF(ISBLANK(A5), "", IF(B5="act", $Q$5, 0))</f>
+        <f t="shared" ref="I5:I13" si="1">IF(ISBLANK(A5), "", IF(B5="act", $Q$5, 0))</f>
         <v>0</v>
       </c>
       <c r="J5" s="12">
-        <f>A5*(1-($Q$4+I5))-((C5-D5)/1000)</f>
+        <f t="shared" ref="J5:J23" si="2">A5*(1-($Q$4+I5))-((C5-D5)/1000)</f>
         <v>833.30000000000007</v>
       </c>
       <c r="K5" s="12">
-        <f>A5*E5/1000</f>
+        <f t="shared" ref="K5:K13" si="3">A5*E5/1000</f>
         <v>0.68</v>
       </c>
       <c r="L5" s="12">
-        <f>IF(ISBLANK(A5), "", J5*G5/1000)</f>
+        <f t="shared" ref="L5:L23" si="4">IF(ISBLANK(A5), "", J5*G5/1000)</f>
         <v>0.67497300000000005</v>
       </c>
       <c r="M5" s="12">
@@ -1012,43 +1011,43 @@
       </c>
       <c r="D6" s="12"/>
       <c r="E6" s="12">
-        <f>IF(ISBLANK(A6), "", VLOOKUP(B6, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.79</v>
       </c>
       <c r="F6" s="12">
-        <f t="shared" ref="F6:F23" si="0">IF(ISBLANK(A6), "", VLOOKUP(B6, $P$20:$T$28, 4, FALSE))</f>
+        <f t="shared" ref="F6:F23" si="5">IF(ISBLANK(A6), "", VLOOKUP(B6, $P$20:$T$28, 4, FALSE))</f>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G6" s="12">
-        <f t="shared" ref="G6:G13" si="1">$Q$15</f>
+        <f t="shared" ref="G6:G13" si="6">$Q$15</f>
         <v>0.81</v>
       </c>
       <c r="H6" s="12">
-        <f t="shared" ref="H6:H23" si="2">$R$15</f>
+        <f t="shared" ref="H6:H23" si="7">$R$15</f>
         <v>0.1</v>
       </c>
       <c r="I6" s="12">
-        <f>IF(ISBLANK(A6), "", IF(B6="act", $Q$5, 0))</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J6" s="12">
-        <f>A6*(1-($Q$4+I6))-((C6-D6)/1000)</f>
+        <f t="shared" si="2"/>
         <v>1666.6000000000001</v>
       </c>
       <c r="K6" s="12">
-        <f>A6*E6/1000</f>
+        <f t="shared" si="3"/>
         <v>1.58</v>
       </c>
       <c r="L6" s="12">
-        <f>IF(ISBLANK(A6), "", J6*G6/1000)</f>
+        <f t="shared" si="4"/>
         <v>1.3499460000000001</v>
       </c>
       <c r="M6" s="12">
-        <f t="shared" ref="M6:M23" si="3">IF(ISBLANK(A6), "", A6*F6/1000)</f>
+        <f t="shared" ref="M6:M23" si="8">IF(ISBLANK(A6), "", A6*F6/1000)</f>
         <v>0.14000000000000001</v>
       </c>
       <c r="N6" s="12">
-        <f t="shared" ref="N6:N23" si="4">IF(ISBLANK(A6), "", J6*H6/1000)</f>
+        <f t="shared" ref="N6:N23" si="9">IF(ISBLANK(A6), "", J6*H6/1000)</f>
         <v>0.16666000000000003</v>
       </c>
       <c r="O6" s="12"/>
@@ -1062,43 +1061,43 @@
       </c>
       <c r="D7" s="12"/>
       <c r="E7" s="12">
-        <f>IF(ISBLANK(A7), "", VLOOKUP(B7, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.73</v>
       </c>
       <c r="F7" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.15</v>
       </c>
       <c r="G7" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H7" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I7" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H7" s="12">
+        <v>0</v>
+      </c>
+      <c r="J7" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I7" s="12">
-        <f>IF(ISBLANK(A7), "", IF(B7="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="12">
-        <f>A7*(1-($Q$4+I7))-((C7-D7)/1000)</f>
         <v>2499.9</v>
       </c>
       <c r="K7" s="12">
-        <f>A7*E7/1000</f>
+        <f t="shared" si="3"/>
         <v>2.19</v>
       </c>
       <c r="L7" s="12">
-        <f>IF(ISBLANK(A7), "", J7*G7/1000)</f>
+        <f t="shared" si="4"/>
         <v>2.0249190000000001</v>
       </c>
       <c r="M7" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.45</v>
       </c>
       <c r="N7" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.24999000000000002</v>
       </c>
       <c r="O7" s="12"/>
@@ -1112,43 +1111,43 @@
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="12">
-        <f>IF(ISBLANK(A8), "", VLOOKUP(B8, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.25</v>
       </c>
       <c r="F8" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.08</v>
       </c>
       <c r="G8" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H8" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I8" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H8" s="12">
+        <v>0</v>
+      </c>
+      <c r="J8" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I8" s="12">
-        <f>IF(ISBLANK(A8), "", IF(B8="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J8" s="12">
-        <f>A8*(1-($Q$4+I8))-((C8-D8)/1000)</f>
         <v>3333.2000000000003</v>
       </c>
       <c r="K8" s="12">
-        <f>A8*E8/1000</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="L8" s="12">
-        <f>IF(ISBLANK(A8), "", J8*G8/1000)</f>
+        <f t="shared" si="4"/>
         <v>2.6998920000000002</v>
       </c>
       <c r="M8" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.32</v>
       </c>
       <c r="N8" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.33332000000000006</v>
       </c>
       <c r="O8" s="12"/>
@@ -1162,43 +1161,43 @@
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="12">
-        <f>IF(ISBLANK(A9), "", VLOOKUP(B9, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.53</v>
       </c>
       <c r="F9" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.04</v>
       </c>
       <c r="G9" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H9" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I9" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H9" s="12">
+        <v>0</v>
+      </c>
+      <c r="J9" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I9" s="12">
-        <f>IF(ISBLANK(A9), "", IF(B9="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="12">
-        <f>A9*(1-($Q$4+I9))-((C9-D9)/1000)</f>
         <v>4166.5</v>
       </c>
       <c r="K9" s="12">
-        <f>A9*E9/1000</f>
+        <f t="shared" si="3"/>
         <v>2.65</v>
       </c>
       <c r="L9" s="12">
-        <f>IF(ISBLANK(A9), "", J9*G9/1000)</f>
+        <f t="shared" si="4"/>
         <v>3.3748650000000002</v>
       </c>
       <c r="M9" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.2</v>
       </c>
       <c r="N9" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.41665000000000002</v>
       </c>
     </row>
@@ -1211,43 +1210,43 @@
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="12">
-        <f>IF(ISBLANK(A10), "", VLOOKUP(B10, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.62</v>
       </c>
       <c r="F10" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G10" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H10" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I10" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H10" s="12">
+        <v>0</v>
+      </c>
+      <c r="J10" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I10" s="12">
-        <f>IF(ISBLANK(A10), "", IF(B10="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="12">
-        <f>A10*(1-($Q$4+I10))-((C10-D10)/1000)</f>
         <v>4999.8</v>
       </c>
       <c r="K10" s="12">
-        <f>A10*E10/1000</f>
+        <f t="shared" si="3"/>
         <v>3.72</v>
       </c>
       <c r="L10" s="12">
-        <f>IF(ISBLANK(A10), "", J10*G10/1000)</f>
+        <f t="shared" si="4"/>
         <v>4.0498380000000003</v>
       </c>
       <c r="M10" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.42000000000000004</v>
       </c>
       <c r="N10" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.49998000000000004</v>
       </c>
     </row>
@@ -1260,43 +1259,43 @@
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="12">
-        <f>IF(ISBLANK(A11), "", VLOOKUP(B11, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.12</v>
       </c>
       <c r="F11" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="G11" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H11" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I11" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H11" s="12">
+        <v>0</v>
+      </c>
+      <c r="J11" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I11" s="12">
-        <f>IF(ISBLANK(A11), "", IF(B11="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="12">
-        <f>A11*(1-($Q$4+I11))-((C11-D11)/1000)</f>
         <v>5833.1</v>
       </c>
       <c r="K11" s="12">
-        <f>A11*E11/1000</f>
+        <f t="shared" si="3"/>
         <v>0.84</v>
       </c>
       <c r="L11" s="12">
-        <f>IF(ISBLANK(A11), "", J11*G11/1000)</f>
+        <f t="shared" si="4"/>
         <v>4.7248110000000008</v>
       </c>
       <c r="M11" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N11" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.58331000000000011</v>
       </c>
     </row>
@@ -1309,43 +1308,43 @@
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="12">
-        <f>IF(ISBLANK(A12), "", VLOOKUP(B12, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.54</v>
       </c>
       <c r="F12" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G12" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H12" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I12" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H12" s="12">
+        <v>0</v>
+      </c>
+      <c r="J12" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I12" s="12">
-        <f>IF(ISBLANK(A12), "", IF(B12="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="12">
-        <f>A12*(1-($Q$4+I12))-((C12-D12)/1000)</f>
         <v>6666.4000000000005</v>
       </c>
       <c r="K12" s="12">
-        <f>A12*E12/1000</f>
+        <f t="shared" si="3"/>
         <v>4.32</v>
       </c>
       <c r="L12" s="12">
-        <f>IF(ISBLANK(A12), "", J12*G12/1000)</f>
+        <f t="shared" si="4"/>
         <v>5.3997840000000004</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="N12" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.66664000000000012</v>
       </c>
     </row>
@@ -1359,43 +1358,43 @@
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
       <c r="E13" s="12">
-        <f>IF(ISBLANK(A13), "", VLOOKUP(B13, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="0"/>
         <v>0.68</v>
       </c>
       <c r="F13" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="G13" s="12">
+        <f t="shared" si="6"/>
+        <v>0.81</v>
+      </c>
+      <c r="H13" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I13" s="12">
         <f t="shared" si="1"/>
-        <v>0.81</v>
-      </c>
-      <c r="H13" s="12">
+        <v>0.74129999999999996</v>
+      </c>
+      <c r="J13" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I13" s="12">
-        <f>IF(ISBLANK(A13), "", IF(B13="act", $Q$5, 0))</f>
-        <v>0.74129999999999996</v>
-      </c>
-      <c r="J13" s="12">
-        <f>A13*(1-($Q$4+I13))-((C13-D13)/1000)</f>
         <v>828.00000000000068</v>
       </c>
       <c r="K13" s="12">
-        <f>A13*E13/1000</f>
+        <f t="shared" si="3"/>
         <v>6.12</v>
       </c>
       <c r="L13" s="12">
-        <f>IF(ISBLANK(A13), "", J13*G13/1000)</f>
+        <f t="shared" si="4"/>
         <v>0.67068000000000061</v>
       </c>
       <c r="M13" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.45</v>
       </c>
       <c r="N13" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>8.2800000000000068E-2</v>
       </c>
       <c r="O13" s="12"/>
@@ -1409,27 +1408,27 @@
       <c r="D14" s="12"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="G14" s="12"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
       <c r="J14" s="12">
-        <f>A14*(1-($Q$4+I14))-((C14-D14)/1000)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K14" s="12"/>
       <c r="L14" s="12" t="str">
-        <f>IF(ISBLANK(A14), "", J14*G14/1000)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="M14" s="12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="N14" s="12" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
       <c r="O14" s="12"/>
@@ -1457,11 +1456,11 @@
         <v>0.2</v>
       </c>
       <c r="E15" s="12">
-        <f>IF(ISBLANK(A15), "", VLOOKUP(B15, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" ref="E15:E23" si="10">IF(ISBLANK(A15), "", VLOOKUP(B15, $P$20:$T$28, 2, FALSE))</f>
         <v>0.68</v>
       </c>
       <c r="F15" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="G15" s="12">
@@ -1469,31 +1468,31 @@
         <v>0.81</v>
       </c>
       <c r="H15" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I15" s="12">
+        <f t="shared" ref="I15:I23" si="11">IF(ISBLANK(A15), "", IF(B15="act", $Q$5, 0))</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I15" s="12">
-        <f>IF(ISBLANK(A15), "", IF(B15="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="12">
-        <f>A15*(1-($Q$4+I15))-((C15-D15)/1000)</f>
         <v>833.29970000000003</v>
       </c>
       <c r="K15" s="12">
-        <f>A15*E15/1000</f>
+        <f t="shared" ref="K15:K23" si="12">A15*E15/1000</f>
         <v>0.68</v>
       </c>
       <c r="L15" s="12">
-        <f>IF(ISBLANK(A15), "", J15*G15/1000)</f>
+        <f t="shared" si="4"/>
         <v>0.67497275700000015</v>
       </c>
       <c r="M15" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.05</v>
       </c>
       <c r="N15" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>8.3329970000000003E-2</v>
       </c>
       <c r="O15" s="12"/>
@@ -1521,43 +1520,43 @@
         <v>200</v>
       </c>
       <c r="E16" s="12">
-        <f>IF(ISBLANK(A16), "", VLOOKUP(B16, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.79</v>
       </c>
       <c r="F16" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G16" s="12">
-        <f t="shared" ref="G16:G23" si="5">$Q$15</f>
+        <f t="shared" ref="G16:G23" si="13">$Q$15</f>
         <v>0.81</v>
       </c>
       <c r="H16" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I16" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J16" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I16" s="12">
-        <f>IF(ISBLANK(A16), "", IF(B16="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J16" s="12">
-        <f>A16*(1-($Q$4+I16))-((C16-D16)/1000)</f>
         <v>1666.3000000000002</v>
       </c>
       <c r="K16" s="12">
-        <f>A16*E16/1000</f>
+        <f t="shared" si="12"/>
         <v>1.58</v>
       </c>
       <c r="L16" s="12">
-        <f>IF(ISBLANK(A16), "", J16*G16/1000)</f>
+        <f t="shared" si="4"/>
         <v>1.3497030000000001</v>
       </c>
       <c r="M16" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="N16" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.16663000000000003</v>
       </c>
       <c r="O16" s="12"/>
@@ -1576,43 +1575,43 @@
         <v>200</v>
       </c>
       <c r="E17" s="12">
-        <f>IF(ISBLANK(A17), "", VLOOKUP(B17, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.73</v>
       </c>
       <c r="F17" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.15</v>
       </c>
       <c r="G17" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H17" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I17" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J17" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I17" s="12">
-        <f>IF(ISBLANK(A17), "", IF(B17="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="12">
-        <f>A17*(1-($Q$4+I17))-((C17-D17)/1000)</f>
         <v>2499.7000000000003</v>
       </c>
       <c r="K17" s="12">
-        <f>A17*E17/1000</f>
+        <f t="shared" si="12"/>
         <v>2.19</v>
       </c>
       <c r="L17" s="12">
-        <f>IF(ISBLANK(A17), "", J17*G17/1000)</f>
+        <f t="shared" si="4"/>
         <v>2.0247570000000001</v>
       </c>
       <c r="M17" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.45</v>
       </c>
       <c r="N17" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.24997000000000003</v>
       </c>
       <c r="O17" s="12"/>
@@ -1631,43 +1630,43 @@
         <v>5</v>
       </c>
       <c r="E18" s="12">
-        <f>IF(ISBLANK(A18), "", VLOOKUP(B18, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.25</v>
       </c>
       <c r="F18" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.08</v>
       </c>
       <c r="G18" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H18" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I18" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I18" s="12">
-        <f>IF(ISBLANK(A18), "", IF(B18="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J18" s="12">
-        <f>A18*(1-($Q$4+I18))-((C18-D18)/1000)</f>
         <v>3333.1950000000002</v>
       </c>
       <c r="K18" s="12">
-        <f>A18*E18/1000</f>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="L18" s="12">
-        <f>IF(ISBLANK(A18), "", J18*G18/1000)</f>
+        <f t="shared" si="4"/>
         <v>2.6998879500000004</v>
       </c>
       <c r="M18" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.32</v>
       </c>
       <c r="N18" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.33331950000000005</v>
       </c>
       <c r="O18" s="12"/>
@@ -1686,43 +1685,43 @@
         <v>900</v>
       </c>
       <c r="E19" s="12">
-        <f>IF(ISBLANK(A19), "", VLOOKUP(B19, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.53</v>
       </c>
       <c r="F19" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.04</v>
       </c>
       <c r="G19" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H19" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I19" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I19" s="12">
-        <f>IF(ISBLANK(A19), "", IF(B19="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="12">
-        <f>A19*(1-($Q$4+I19))-((C19-D19)/1000)</f>
         <v>4166.3909999999996</v>
       </c>
       <c r="K19" s="12">
-        <f>A19*E19/1000</f>
+        <f t="shared" si="12"/>
         <v>2.65</v>
       </c>
       <c r="L19" s="12">
-        <f>IF(ISBLANK(A19), "", J19*G19/1000)</f>
+        <f t="shared" si="4"/>
         <v>3.3747767099999999</v>
       </c>
       <c r="M19" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.2</v>
       </c>
       <c r="N19" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.41663909999999998</v>
       </c>
       <c r="O19" s="12"/>
@@ -1757,43 +1756,43 @@
         <v>100</v>
       </c>
       <c r="E20" s="12">
-        <f>IF(ISBLANK(A20), "", VLOOKUP(B20, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.62</v>
       </c>
       <c r="F20" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G20" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H20" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I20" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I20" s="12">
-        <f>IF(ISBLANK(A20), "", IF(B20="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="12">
-        <f>A20*(1-($Q$4+I20))-((C20-D20)/1000)</f>
         <v>4999.7</v>
       </c>
       <c r="K20" s="12">
-        <f>A20*E20/1000</f>
+        <f t="shared" si="12"/>
         <v>3.72</v>
       </c>
       <c r="L20" s="12">
-        <f>IF(ISBLANK(A20), "", J20*G20/1000)</f>
+        <f t="shared" si="4"/>
         <v>4.0497570000000005</v>
       </c>
       <c r="M20" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.42000000000000004</v>
       </c>
       <c r="N20" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.49997000000000003</v>
       </c>
       <c r="O20" s="12"/>
@@ -1827,43 +1826,43 @@
         <v>200</v>
       </c>
       <c r="E21" s="12">
-        <f>IF(ISBLANK(A21), "", VLOOKUP(B21, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.12</v>
       </c>
       <c r="F21" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.01</v>
       </c>
       <c r="G21" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H21" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I21" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I21" s="12">
-        <f>IF(ISBLANK(A21), "", IF(B21="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="12">
-        <f>A21*(1-($Q$4+I21))-((C21-D21)/1000)</f>
         <v>5833</v>
       </c>
       <c r="K21" s="12">
-        <f>A21*E21/1000</f>
+        <f t="shared" si="12"/>
         <v>0.84</v>
       </c>
       <c r="L21" s="12">
-        <f>IF(ISBLANK(A21), "", J21*G21/1000)</f>
+        <f t="shared" si="4"/>
         <v>4.7247300000000001</v>
       </c>
       <c r="M21" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N21" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.58330000000000004</v>
       </c>
       <c r="O21" s="12"/>
@@ -1897,43 +1896,43 @@
         <v>20</v>
       </c>
       <c r="E22" s="12">
-        <f>IF(ISBLANK(A22), "", VLOOKUP(B22, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.54</v>
       </c>
       <c r="F22" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G22" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H22" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I22" s="12">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="J22" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I22" s="12">
-        <f>IF(ISBLANK(A22), "", IF(B22="act", $Q$5, 0))</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="12">
-        <f>A22*(1-($Q$4+I22))-((C22-D22)/1000)</f>
         <v>6666.02</v>
       </c>
       <c r="K22" s="12">
-        <f>A22*E22/1000</f>
+        <f t="shared" si="12"/>
         <v>4.32</v>
       </c>
       <c r="L22" s="12">
-        <f>IF(ISBLANK(A22), "", J22*G22/1000)</f>
+        <f t="shared" si="4"/>
         <v>5.3994762000000014</v>
       </c>
       <c r="M22" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="N22" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>0.66660200000000014</v>
       </c>
       <c r="P22" s="17" t="s">
@@ -1966,43 +1965,43 @@
         <v>200</v>
       </c>
       <c r="E23" s="12">
-        <f>IF(ISBLANK(A23), "", VLOOKUP(B23, $P$20:$T$28, 2, FALSE))</f>
+        <f t="shared" si="10"/>
         <v>0.68</v>
       </c>
       <c r="F23" s="12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="5"/>
         <v>0.05</v>
       </c>
       <c r="G23" s="12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="13"/>
         <v>0.81</v>
       </c>
       <c r="H23" s="12">
+        <f t="shared" si="7"/>
+        <v>0.1</v>
+      </c>
+      <c r="I23" s="12">
+        <f t="shared" si="11"/>
+        <v>0.74129999999999996</v>
+      </c>
+      <c r="J23" s="12">
         <f t="shared" si="2"/>
-        <v>0.1</v>
-      </c>
-      <c r="I23" s="12">
-        <f>IF(ISBLANK(A23), "", IF(B23="act", $Q$5, 0))</f>
-        <v>0.74129999999999996</v>
-      </c>
-      <c r="J23" s="12">
-        <f>A23*(1-($Q$4+I23))-((C23-D23)/1000)</f>
         <v>827.70000000000073</v>
       </c>
       <c r="K23" s="12">
-        <f>A23*E23/1000</f>
+        <f t="shared" si="12"/>
         <v>6.12</v>
       </c>
       <c r="L23" s="12">
-        <f>IF(ISBLANK(A23), "", J23*G23/1000)</f>
+        <f t="shared" si="4"/>
         <v>0.67043700000000062</v>
       </c>
       <c r="M23" s="12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>0.45</v>
       </c>
       <c r="N23" s="12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="9"/>
         <v>8.277000000000008E-2</v>
       </c>
       <c r="P23" s="17" t="s">
@@ -2156,10 +2155,7 @@
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
       <c r="F33" s="12"/>
-      <c r="G33" s="12">
-        <f>(1-($Q$4+$Q$5))</f>
-        <v>9.2000000000000082E-2</v>
-      </c>
+      <c r="G33" s="12"/>
       <c r="H33" s="12"/>
       <c r="I33" s="12"/>
       <c r="J33" s="12"/>
@@ -2176,10 +2172,7 @@
       <c r="D34" s="12"/>
       <c r="E34" s="12"/>
       <c r="F34" s="12"/>
-      <c r="G34" s="12">
-        <f>(A15*(1-($Q$4+$Q$5)))</f>
-        <v>92.000000000000085</v>
-      </c>
+      <c r="G34" s="12"/>
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12"/>
@@ -2194,11 +2187,8 @@
       <c r="D35" s="12"/>
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
-      <c r="G35" s="20">
-        <f>((C15-D15)/1000)</f>
-        <v>2.9999999999999997E-4</v>
-      </c>
-      <c r="H35" s="20"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
       <c r="I35" s="12"/>
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
@@ -2215,10 +2205,7 @@
       <c r="D36" s="12"/>
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
-      <c r="G36" s="12">
-        <f>(A15*(1-($Q$4+$Q$5))-((C15-D15)/1000))*G15/1000</f>
-        <v>7.4519757000000089E-2</v>
-      </c>
+      <c r="G36" s="12"/>
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>

</xml_diff>